<commit_message>
Finished autoconvert training datasets
</commit_message>
<xml_diff>
--- a/src/2023_zf_ovary_re_validation.xlsx
+++ b/src/2023_zf_ovary_re_validation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\其他電腦\My Computer\GlycoMSParser\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F75D9D1E-D2D3-483D-B35D-61CFFD882D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1CB026-34D5-4B04-B8B3-9CDD7F5499A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10350" yWindow="1800" windowWidth="18450" windowHeight="13515" activeTab="1" xr2:uid="{67B4FEEB-0D84-F241-9CC2-FB10DE711B8D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{67B4FEEB-0D84-F241-9CC2-FB10DE711B8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Glycanlist" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="666" uniqueCount="192">
   <si>
     <t>Glycan no (in paper)</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -782,6 +782,10 @@
   </si>
   <si>
     <t>Structure</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>It's F2H7N4S1 (found in 20240922)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1139,9 +1143,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 佈景主題">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主題">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1179,7 +1183,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1285,7 +1289,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1427,7 +1431,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4400,46 +4404,49 @@
         <v>52</v>
       </c>
     </row>
-    <row r="62" spans="1:15">
-      <c r="C62" t="s">
+    <row r="62" spans="1:15" s="9" customFormat="1">
+      <c r="C62" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D62">
+      <c r="D62" s="9">
         <f t="shared" si="16"/>
         <v>3187.5868</v>
       </c>
-      <c r="E62">
+      <c r="E62" s="9">
         <v>3165.6048999999998</v>
       </c>
-      <c r="F62">
+      <c r="F62" s="9">
         <f t="shared" si="17"/>
         <v>1583.3061</v>
       </c>
-      <c r="G62">
+      <c r="G62" s="9">
         <f t="shared" si="18"/>
         <v>1055.8731666666665</v>
       </c>
-      <c r="H62">
+      <c r="H62" s="9">
         <f t="shared" si="0"/>
         <v>792.1567</v>
       </c>
-      <c r="I62">
-        <v>-1</v>
-      </c>
-      <c r="J62">
-        <v>-1</v>
-      </c>
-      <c r="K62">
-        <v>0</v>
-      </c>
-      <c r="L62">
+      <c r="I62" s="9">
+        <v>-1</v>
+      </c>
+      <c r="J62" s="9">
+        <v>-1</v>
+      </c>
+      <c r="K62" s="9">
+        <v>0</v>
+      </c>
+      <c r="L62" s="9">
         <v>6</v>
       </c>
-      <c r="M62">
-        <v>-1</v>
-      </c>
-      <c r="N62" t="s">
+      <c r="M62" s="9">
+        <v>-1</v>
+      </c>
+      <c r="N62" s="9" t="s">
         <v>53</v>
+      </c>
+      <c r="O62" s="9" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="63" spans="1:15">
@@ -4789,7 +4796,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACF3915D-BEE4-3D4E-9D03-D3E2CBF59D16}">
-  <dimension ref="A1:E263"/>
+  <dimension ref="A1:E257"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="20.125" customWidth="1"/>
@@ -9133,10 +9140,10 @@
     </row>
     <row r="256" spans="1:5">
       <c r="A256" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
       <c r="B256">
-        <v>22603</v>
+        <v>24019</v>
       </c>
       <c r="C256">
         <v>1</v>
@@ -9145,15 +9152,15 @@
         <v>3</v>
       </c>
       <c r="E256">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="257" spans="1:5">
       <c r="A257" t="s">
-        <v>147</v>
+        <v>170</v>
       </c>
       <c r="B257">
-        <v>22807</v>
+        <v>29349</v>
       </c>
       <c r="C257">
         <v>1</v>
@@ -9162,108 +9169,6 @@
         <v>3</v>
       </c>
       <c r="E257">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="258" spans="1:5">
-      <c r="A258" t="s">
-        <v>147</v>
-      </c>
-      <c r="B258">
-        <v>23140</v>
-      </c>
-      <c r="C258">
-        <v>1</v>
-      </c>
-      <c r="D258">
-        <v>3</v>
-      </c>
-      <c r="E258">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="259" spans="1:5">
-      <c r="A259" t="s">
-        <v>147</v>
-      </c>
-      <c r="B259">
-        <v>23979</v>
-      </c>
-      <c r="C259">
-        <v>2</v>
-      </c>
-      <c r="D259">
-        <v>3</v>
-      </c>
-      <c r="E259">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="260" spans="1:5">
-      <c r="A260" t="s">
-        <v>147</v>
-      </c>
-      <c r="B260">
-        <v>24163</v>
-      </c>
-      <c r="C260">
-        <v>2</v>
-      </c>
-      <c r="D260">
-        <v>3</v>
-      </c>
-      <c r="E260">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="261" spans="1:5">
-      <c r="A261" t="s">
-        <v>147</v>
-      </c>
-      <c r="B261">
-        <v>24383</v>
-      </c>
-      <c r="C261">
-        <v>2</v>
-      </c>
-      <c r="D261">
-        <v>3</v>
-      </c>
-      <c r="E261">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="262" spans="1:5">
-      <c r="A262" t="s">
-        <v>166</v>
-      </c>
-      <c r="B262">
-        <v>24019</v>
-      </c>
-      <c r="C262">
-        <v>1</v>
-      </c>
-      <c r="D262">
-        <v>3</v>
-      </c>
-      <c r="E262">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="263" spans="1:5">
-      <c r="A263" t="s">
-        <v>170</v>
-      </c>
-      <c r="B263">
-        <v>29349</v>
-      </c>
-      <c r="C263">
-        <v>1</v>
-      </c>
-      <c r="D263">
-        <v>3</v>
-      </c>
-      <c r="E263">
         <v>2</v>
       </c>
     </row>

</xml_diff>